<commit_message>
Added:     devnet_line_plot new plotting script to visualize line deration impacts     Option in devnet_menu.py for the new script.     Documentation in README.md Included:     DevNet Stress Report_5.html     line_vs_metrics.png     devnet_plots.xlsx     devnet_stress_tc.md
</commit_message>
<xml_diff>
--- a/denvnet-stress-vectors/devnet_plots.xlsx
+++ b/denvnet-stress-vectors/devnet_plots.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeronode-my.sharepoint.com/personal/ashok_zeronode_ca/Documents/Ashok/SFU- SustainableEnergyEngineering/Sustainable Energy &amp; Datacenter Models Tools/EnergySystemAnalysis- PyPSA/pypsa-asr/denvnet-stress-vectors/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeronode-my.sharepoint.com/personal/ashok_zeronode_ca/Documents/Ashok/SFU- SustainableEnergyEngineering/Sustainable Energy &amp; Datacenter Models Tools/EnergySystemAnalysis- PyPSA/pypsa-zn/denvnet-stress-vectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{1DE9AB68-969B-4576-8842-DCCCDAC6DEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{035701C4-2AE7-457E-840A-0659A4DA794D}"/>
+  <xr:revisionPtr revIDLastSave="284" documentId="8_{1DE9AB68-969B-4576-8842-DCCCDAC6DEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86AAF940-6173-4F6D-AD88-3C873BD4FC2B}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="1" xr2:uid="{7340CB05-3689-448E-B208-BC226AF7FE68}"/>
+    <workbookView xWindow="28680" yWindow="-12165" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{7340CB05-3689-448E-B208-BC226AF7FE68}"/>
   </bookViews>
   <sheets>
     <sheet name="DevNetGen_mc&lt;&gt;LMP" sheetId="1" r:id="rId1"/>
     <sheet name="DevNet_load&lt;&gt;SystemCost" sheetId="2" r:id="rId2"/>
+    <sheet name="DevNet_line&lt;&gt;near_bind_ct" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="76">
   <si>
     <t>case</t>
   </si>
@@ -224,15 +225,6 @@
     <t>DevNet base params:</t>
   </si>
   <si>
-    <t xml:space="preserve">  Buses_N            =</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  c_g (USD/MWh)      =</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  line s_nom (MW)    =</t>
-  </si>
-  <si>
     <t>Total System Load
 (MW)</t>
   </si>
@@ -247,6 +239,61 @@
   </si>
   <si>
     <t>DevNet Stress Report_5.html</t>
+  </si>
+  <si>
+    <t>c17</t>
+  </si>
+  <si>
+    <t>c18</t>
+  </si>
+  <si>
+    <t>c19</t>
+  </si>
+  <si>
+    <t>c20</t>
+  </si>
+  <si>
+    <t>c21</t>
+  </si>
+  <si>
+    <t>c22</t>
+  </si>
+  <si>
+    <t>k_line_WECC_NW</t>
+  </si>
+  <si>
+    <t>k_line_WECC_SW</t>
+  </si>
+  <si>
+    <t>k_line_SPP_MISO</t>
+  </si>
+  <si>
+    <t>k_line_PJM_NE</t>
+  </si>
+  <si>
+    <t>k_line_SERC_SE</t>
+  </si>
+  <si>
+    <t>k_line_ERCOT</t>
+  </si>
+  <si>
+    <t>Bus_{Load}</t>
+  </si>
+  <si>
+    <t>=</t>
+  </si>
+  <si>
+    <t>Buses_N</t>
+  </si>
+  <si>
+    <t>c_g (USD/MWh)</t>
+  </si>
+  <si>
+    <t>line s_nom (MW)</t>
+  </si>
+  <si>
+    <t>Each line effective
+(MW)</t>
   </si>
 </sst>
 </file>
@@ -336,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -374,20 +421,20 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3626,10 +3673,10 @@
     </row>
     <row r="3" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="2:20" x14ac:dyDescent="0.3">
@@ -4278,25 +4325,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D410345-51F7-4EF5-A7EE-15839BFCDB90}">
-  <dimension ref="B1:O16"/>
+  <dimension ref="B2:O16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="10.77734375" customWidth="1"/>
-    <col min="4" max="15" width="20.77734375" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="3" width="10.77734375" style="1" customWidth="1"/>
+    <col min="4" max="15" width="20.77734375" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15" s="1" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="2:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -4308,35 +4356,44 @@
       </c>
     </row>
     <row r="5" spans="2:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="13" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="4"/>
     </row>
     <row r="6" spans="2:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="17" t="s">
-        <v>53</v>
+      <c r="B6" s="13" t="s">
+        <v>72</v>
       </c>
       <c r="C6" s="4"/>
-      <c r="E6" s="20">
+      <c r="D6" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="14">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="2:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="17" t="s">
-        <v>54</v>
+      <c r="B7" s="13" t="s">
+        <v>73</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="E7" s="18">
+      <c r="D7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="8">
         <v>50</v>
       </c>
     </row>
     <row r="8" spans="2:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="17" t="s">
-        <v>55</v>
+      <c r="B8" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="E8" s="20">
+      <c r="D8" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" s="14">
         <v>5000</v>
       </c>
     </row>
@@ -4370,10 +4427,10 @@
         <v>44</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="L10" s="15" t="s">
         <v>45</v>
@@ -4389,278 +4446,278 @@
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="7">
         <v>1</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="7">
         <v>1</v>
       </c>
-      <c r="F11" s="14">
+      <c r="F11" s="7">
         <v>1</v>
       </c>
-      <c r="G11" s="14">
+      <c r="G11" s="7">
         <v>1</v>
       </c>
-      <c r="H11" s="14">
+      <c r="H11" s="7">
         <v>1</v>
       </c>
-      <c r="I11" s="14">
+      <c r="I11" s="7">
         <v>1</v>
       </c>
-      <c r="J11" s="19">
+      <c r="J11" s="16">
         <f>SUM((D11*$E$8) + (E11*$E$8) + (F11*$E$8) + (G11*$E$8) + (H11*$E$8) + (I11*$E$8))</f>
         <v>30000</v>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="16">
         <f>$E$7*J11</f>
         <v>1500000</v>
       </c>
-      <c r="L11" s="16">
+      <c r="L11" s="8">
         <v>1500000</v>
       </c>
-      <c r="M11" s="16">
+      <c r="M11" s="8">
         <v>0</v>
       </c>
-      <c r="N11" s="14">
+      <c r="N11" s="7">
         <v>1</v>
       </c>
-      <c r="O11" s="16">
+      <c r="O11" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="7">
         <v>1.2</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="7">
         <v>1.2</v>
       </c>
-      <c r="F12" s="14">
+      <c r="F12" s="7">
         <v>1.2</v>
       </c>
-      <c r="G12" s="14">
+      <c r="G12" s="7">
         <v>1.2</v>
       </c>
-      <c r="H12" s="14">
+      <c r="H12" s="7">
         <v>1.2</v>
       </c>
-      <c r="I12" s="14">
+      <c r="I12" s="7">
         <v>1.2</v>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="16">
         <f t="shared" ref="J12:J16" si="0">SUM((D12*$E$8) + (E12*$E$8) + (F12*$E$8) + (G12*$E$8) + (H12*$E$8) + (I12*$E$8))</f>
         <v>36000</v>
       </c>
-      <c r="K12" s="19">
+      <c r="K12" s="16">
         <f t="shared" ref="K12:K16" si="1">$E$7*J12</f>
         <v>1800000</v>
       </c>
-      <c r="L12" s="16">
+      <c r="L12" s="8">
         <v>1800000</v>
       </c>
-      <c r="M12" s="16">
+      <c r="M12" s="8">
         <v>0</v>
       </c>
-      <c r="N12" s="14">
+      <c r="N12" s="7">
         <v>0.8</v>
       </c>
-      <c r="O12" s="16">
+      <c r="O12" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="7">
         <v>1.4</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="7">
         <v>1.4</v>
       </c>
-      <c r="F13" s="14">
+      <c r="F13" s="7">
         <v>1.4</v>
       </c>
-      <c r="G13" s="14">
+      <c r="G13" s="7">
         <v>1.4</v>
       </c>
-      <c r="H13" s="14">
+      <c r="H13" s="7">
         <v>1.4</v>
       </c>
-      <c r="I13" s="14">
+      <c r="I13" s="7">
         <v>1.4</v>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="16">
         <f t="shared" si="0"/>
         <v>42000</v>
       </c>
-      <c r="K13" s="19">
+      <c r="K13" s="16">
         <f t="shared" si="1"/>
         <v>2100000</v>
       </c>
-      <c r="L13" s="16">
+      <c r="L13" s="8">
         <v>2100000</v>
       </c>
-      <c r="M13" s="16">
+      <c r="M13" s="8">
         <v>0</v>
       </c>
-      <c r="N13" s="14">
+      <c r="N13" s="7">
         <v>0.5</v>
       </c>
-      <c r="O13" s="16">
+      <c r="O13" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="7">
         <v>1.6</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="7">
         <v>1.6</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="7">
         <v>1.6</v>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="7">
         <v>1.6</v>
       </c>
-      <c r="H14" s="14">
+      <c r="H14" s="7">
         <v>1.6</v>
       </c>
-      <c r="I14" s="14">
+      <c r="I14" s="7">
         <v>1.6</v>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="16">
         <f t="shared" si="0"/>
         <v>48000</v>
       </c>
-      <c r="K14" s="19">
+      <c r="K14" s="16">
         <f t="shared" si="1"/>
         <v>2400000</v>
       </c>
-      <c r="L14" s="16">
+      <c r="L14" s="8">
         <v>2400000</v>
       </c>
-      <c r="M14" s="16">
+      <c r="M14" s="8">
         <v>0</v>
       </c>
-      <c r="N14" s="14">
+      <c r="N14" s="7">
         <v>0</v>
       </c>
-      <c r="O14" s="16">
+      <c r="O14" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="7">
         <v>1.8</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="7">
         <v>1.8</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="7">
         <v>1.8</v>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="7">
         <v>1.8</v>
       </c>
-      <c r="H15" s="14">
+      <c r="H15" s="7">
         <v>1.8</v>
       </c>
-      <c r="I15" s="14">
+      <c r="I15" s="7">
         <v>1.8</v>
       </c>
-      <c r="J15" s="19">
+      <c r="J15" s="16">
         <f t="shared" si="0"/>
         <v>54000</v>
       </c>
-      <c r="K15" s="19">
+      <c r="K15" s="16">
         <f t="shared" si="1"/>
         <v>2700000</v>
       </c>
-      <c r="L15" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="M15" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="N15" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="O15" s="16">
+      <c r="L15" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="M15" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="O15" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="7">
         <v>2</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="7">
         <v>2</v>
       </c>
-      <c r="F16" s="14">
+      <c r="F16" s="7">
         <v>2</v>
       </c>
-      <c r="G16" s="14">
+      <c r="G16" s="7">
         <v>2</v>
       </c>
-      <c r="H16" s="14">
+      <c r="H16" s="7">
         <v>2</v>
       </c>
-      <c r="I16" s="14">
+      <c r="I16" s="7">
         <v>2</v>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="16">
         <f t="shared" si="0"/>
         <v>60000</v>
       </c>
-      <c r="K16" s="19">
+      <c r="K16" s="16">
         <f t="shared" si="1"/>
         <v>3000000</v>
       </c>
-      <c r="L16" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="M16" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="N16" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="O16" s="16">
+      <c r="L16" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="M16" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="O16" s="8">
         <v>0</v>
       </c>
     </row>
@@ -4668,4 +4725,615 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2FCF0BC-771C-4579-B778-06B9A363C61B}">
+  <dimension ref="B2:V21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="3" width="10.77734375" style="1" customWidth="1"/>
+    <col min="4" max="12" width="20.77734375" style="1" customWidth="1"/>
+    <col min="13" max="16" width="15.77734375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="25.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="20.77734375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="25.77734375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="20.77734375" style="1" customWidth="1"/>
+    <col min="21" max="21" width="25.77734375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="20.77734375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="1.77734375" style="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="2:22" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="2:22" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="2:22" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="14">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="8" spans="2:22" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" s="8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="2:22" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="14">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="10" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B10" s="3"/>
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="2:22" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B11" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="M11" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="N11" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="O11" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="P11" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="T11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="U11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="V11" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="7">
+        <v>1</v>
+      </c>
+      <c r="E12" s="7">
+        <v>1</v>
+      </c>
+      <c r="F12" s="7">
+        <v>1</v>
+      </c>
+      <c r="G12" s="7">
+        <v>1</v>
+      </c>
+      <c r="H12" s="7">
+        <v>1</v>
+      </c>
+      <c r="I12" s="7">
+        <v>1</v>
+      </c>
+      <c r="J12" s="16">
+        <f>AVERAGE(D12:I12)*$E$9</f>
+        <v>5000</v>
+      </c>
+      <c r="K12" s="16">
+        <f>$E$6*$E$7</f>
+        <v>30000</v>
+      </c>
+      <c r="L12" s="16">
+        <f>$E$8*K12</f>
+        <v>1500000</v>
+      </c>
+      <c r="M12" s="8">
+        <v>1500000</v>
+      </c>
+      <c r="N12" s="8">
+        <v>0</v>
+      </c>
+      <c r="O12" s="7">
+        <v>1</v>
+      </c>
+      <c r="P12" s="8">
+        <v>2</v>
+      </c>
+      <c r="Q12" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="R12" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="S12" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="T12" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="U12" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="V12" s="12">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="13" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="E13" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="F13" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="G13" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="H13" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="I13" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="J13" s="16">
+        <f t="shared" ref="J13:J17" si="0">AVERAGE(D13:I13)*$E$9</f>
+        <v>3999.9999999999995</v>
+      </c>
+      <c r="K13" s="16">
+        <f t="shared" ref="K13:K17" si="1">$E$6*$E$7</f>
+        <v>30000</v>
+      </c>
+      <c r="L13" s="16">
+        <f t="shared" ref="L13:L17" si="2">$E$8*K13</f>
+        <v>1500000</v>
+      </c>
+      <c r="M13" s="8">
+        <v>1500000</v>
+      </c>
+      <c r="N13" s="8">
+        <v>0</v>
+      </c>
+      <c r="O13" s="7">
+        <v>1</v>
+      </c>
+      <c r="P13" s="8">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="R13" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="S13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="T13" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="U13" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="V13" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="E14" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="F14" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="G14" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="H14" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="I14" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="J14" s="16">
+        <f t="shared" si="0"/>
+        <v>3000</v>
+      </c>
+      <c r="K14" s="16">
+        <f t="shared" si="1"/>
+        <v>30000</v>
+      </c>
+      <c r="L14" s="16">
+        <f t="shared" si="2"/>
+        <v>1500000</v>
+      </c>
+      <c r="M14" s="8">
+        <v>1500000</v>
+      </c>
+      <c r="N14" s="8">
+        <v>0</v>
+      </c>
+      <c r="O14" s="7">
+        <v>1</v>
+      </c>
+      <c r="P14" s="8">
+        <v>4</v>
+      </c>
+      <c r="Q14" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="R14" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="S14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="T14" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="U14" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="V14" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B15" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="E15" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="F15" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="G15" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="H15" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="I15" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="J15" s="16">
+        <f t="shared" si="0"/>
+        <v>1999.9999999999998</v>
+      </c>
+      <c r="K15" s="16">
+        <f t="shared" si="1"/>
+        <v>30000</v>
+      </c>
+      <c r="L15" s="16">
+        <f t="shared" si="2"/>
+        <v>1500000</v>
+      </c>
+      <c r="M15" s="8">
+        <v>1500000</v>
+      </c>
+      <c r="N15" s="8">
+        <v>0</v>
+      </c>
+      <c r="O15" s="7">
+        <v>1</v>
+      </c>
+      <c r="P15" s="8">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="R15" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="S15" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="T15" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="U15" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="V15" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="E16" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="F16" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="G16" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="H16" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="I16" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="J16" s="16">
+        <f t="shared" si="0"/>
+        <v>999.99999999999989</v>
+      </c>
+      <c r="K16" s="16">
+        <f t="shared" si="1"/>
+        <v>30000</v>
+      </c>
+      <c r="L16" s="16">
+        <f t="shared" si="2"/>
+        <v>1500000</v>
+      </c>
+      <c r="M16" s="17">
+        <v>1500000</v>
+      </c>
+      <c r="N16" s="17">
+        <v>0</v>
+      </c>
+      <c r="O16" s="12">
+        <v>1</v>
+      </c>
+      <c r="P16" s="8">
+        <v>6</v>
+      </c>
+      <c r="Q16" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="R16" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="S16" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="T16" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="U16" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="V16" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="F17" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="G17" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="H17" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="I17" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="J17" s="16">
+        <f t="shared" si="0"/>
+        <v>499.99999999999994</v>
+      </c>
+      <c r="K17" s="16">
+        <f t="shared" si="1"/>
+        <v>30000</v>
+      </c>
+      <c r="L17" s="16">
+        <f t="shared" si="2"/>
+        <v>1500000</v>
+      </c>
+      <c r="M17" s="17">
+        <v>1500000</v>
+      </c>
+      <c r="N17" s="17">
+        <v>0</v>
+      </c>
+      <c r="O17" s="12">
+        <v>1</v>
+      </c>
+      <c r="P17" s="8">
+        <v>6</v>
+      </c>
+      <c r="Q17" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="R17" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="S17" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="T17" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="U17" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="V17" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
+    </row>
+    <row r="19" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="Q19"/>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19"/>
+      <c r="V19"/>
+    </row>
+    <row r="20" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+    </row>
+    <row r="21" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="Q21"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21"/>
+      <c r="V21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="R12:V17" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>